<commit_message>
[WI-TEST] Vòng chạy đầy đủ 76 ca sau sáu đợt sửa — 11 Đạt, 57 Không đạt, 8 Bị chặn (16%)
Chấm lại toàn bộ trên vòng chạy đầy đủ, không giữ phán quyết của các lần chạy
lẻ. Hai ca KHÔNG ỔN ĐỊNH giữa các lần chạy được ghi riêng thay vì chấm theo
lần đẹp nhất:

  TC004 — unknown → 4 câu hỏi đúng bài toán; project.create → dự án lồng + hỏi ISA
  TC043 — lần nạp được tệp và trả lời đúng; lần E5002 vì slots.path không được
          điền. Cùng lần chạy, TC042 (câu cùng hình dạng) lại nạp được.

TC005 → Đạt: chỉ ra mâu thuẫn BẰNG SỐ (CR2032 220mAh không cấp nổi cho 4K),
nhờ DEV-206 cho req.elicit hỏi cả gaps.

Không ca nào treo; chậm nhất 95,5 s (vòng đầu có ca 904 s).

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Usecase_Test_Agent_Ky_Su_Nhung.xlsx
+++ b/docs/Usecase_Test_Agent_Ky_Su_Nhung.xlsx
@@ -2113,12 +2113,12 @@
       </c>
       <c r="I5" s="26" t="inlineStr">
         <is>
-          <t>Đạt</t>
+          <t>Không đạt</t>
         </is>
       </c>
       <c r="J5" s="26" t="inlineStr">
         <is>
-          <t>Không bịa yêu cầu, không sinh thiết kế nào. Có đặt câu hỏi làm rõ VỀ BÀI TOÁN: “Chưa rõ yêu cầu về kết nối mạng (Wi-Fi, Bluetooth, Zigbee, LoRa)”.</t>
+          <t>KHÔNG ỔN ĐỊNH. Khi `parse_intent` cho ra `unknown` thì tác tử hỏi BỐN câu về chính bài toán (“Mạch thông minh này cụ thể dùng để làm gì?”, “Nguồn cấp là gì?”, “Môi trường hoạt động?”) — đúng đề bài. Khi nó cho ra `project.create` (lần chạy đầy đủ 23/09) thì tạo một dự án LỒNG `mach-thong-minh/cai-mach-thong-minh` rồi hỏi ISA.</t>
         </is>
       </c>
       <c r="K5" s="26" t="inlineStr">
@@ -2133,7 +2133,7 @@
       </c>
       <c r="M5" s="26" t="inlineStr">
         <is>
-          <t>Điểm trừ: câu hỏi ấy viết KHÔNG DẤU (“Chua ro yeu cau ve ket noi mang”) trong một sản phẩm tiếng Việt; và hai câu hỏi còn lại vẫn là tham số (`reqset_ids`, `style`).</t>
+          <t>Chấm theo lần chạy đầy đủ, không theo lần chạy đẹp nhất. Hai nhánh ý định cho hai hành vi khác hẳn nhau cho cùng một câu — đây là chỗ cần chạy lặp 3–5 lần như sheet Huong dan đòi, chứ không phải chỗ chốt bằng một lần.</t>
         </is>
       </c>
     </row>
@@ -2180,12 +2180,12 @@
       </c>
       <c r="I6" s="26" t="inlineStr">
         <is>
-          <t>Không đạt</t>
+          <t>Đạt</t>
         </is>
       </c>
       <c r="J6" s="26" t="inlineStr">
         <is>
-          <t>Rút ra hai yêu cầu có số liệu tốt (4K 24 fps độ trễ &lt; 200 ms qua LoRa; 43 800 giờ trên pin CR2032 220 mAh ⇒ ≤ 5 µA) và tự đánh dấu một yêu cầu “✖ KHÔNG ĐO ĐƯỢC”. Nhưng KHÔNG hề nói hai yêu cầu ấy mâu thuẫn nhau và bất khả thi vật lý; báo “✅ Xong 6/6 bước”.</t>
+          <t>SAU [DEV-206]: chỉ ra mâu thuẫn BẰNG SỐ — “Pin nút áo (ví dụ CR2032) chỉ có dung lượng khoảng 220mAh, không thể cấp nguồn cho cảm biến 4K và vi điều khiển xử lý video liên tục”. Kèm 5 điểm cần làm rõ (môi trường, khả thi/nguồn…). Không đưa ra thiết kế giả vờ khả thi.</t>
         </is>
       </c>
       <c r="K6" s="26" t="inlineStr">
@@ -2200,7 +2200,7 @@
       </c>
       <c r="M6" s="26" t="inlineStr">
         <is>
-          <t>Điểm cộng: không đưa ra thiết kế giả vờ khả thi. `req.detect_conflict` có chạy nhưng không bắt được mâu thuẫn băng thông/năng lượng.</t>
+          <t>Đúng chữ đề bài chờ: “chỉ ra mâu thuẫn bằng số liệu… đề xuất nới ràng buộc nào”. Trước [DEV-206] `req.elicit` trả 0 gaps nên không có chỗ nào nói ra điều này.</t>
         </is>
       </c>
     </row>
@@ -4650,12 +4650,12 @@
       </c>
       <c r="I44" s="26" t="inlineStr">
         <is>
-          <t>Đạt</t>
+          <t>Không đạt</t>
         </is>
       </c>
       <c r="J44" s="26" t="inlineStr">
         <is>
-          <t>SAU [DEV-202]: “Thông tin về dải nhiệt độ hoạt động của MCU-X không có trong đoạn văn được cung cấp [1].” Đọc tài liệu thật, tìm không thấy, nói ra, kèm trích dẫn.</t>
+          <t>KHÔNG ỔN ĐỊNH. Lần chạy riêng: đọc tài liệu và trả lời đúng “không có trong đoạn văn được cung cấp [1]”. Lần chạy đầy đủ 23/09: `view.rag_ask` hỏng E5002 “dự án chưa có tài liệu nào” — tệp trong câu KHÔNG được nạp.</t>
         </is>
       </c>
       <c r="K44" s="26" t="inlineStr">
@@ -4670,7 +4670,7 @@
       </c>
       <c r="M44" s="26" t="inlineStr">
         <is>
-          <t>Trước đây ca này cũng KHÔNG bịa — nhưng vì tài liệu chưa bao giờ được đọc, nên phép đo ấy vô nghĩa. Giờ tính chất chống bịa được chứng minh THẬT: tài liệu đã nạp (3 đoạn), tác tử tra và trả lời rằng không có.</t>
+          <t>Nguyên nhân: `${_path}` phụ thuộc `chat.parse_intent` điền `slots.path`, mà việc ấy không tất định. Cùng lần chạy, TC042 (câu cùng hình dạng) lại nạp được và trả lời đúng kèm trang 412. Cần rút đường dẫn XÁC ĐỊNH từ câu chữ, không nhờ mô hình.</t>
         </is>
       </c>
     </row>
@@ -6045,7 +6045,7 @@
       </c>
       <c r="J66" s="26" t="inlineStr">
         <is>
-          <t>Mở lại dự án rồi hỏi “Tiếp tục dự án này, trước đó đã chốt những gì?” — tác tử hỏi ngược “id hoặc đường dẫn” của dự án, dù dự án ĐANG MỞ. Không khôi phục được quyết định nào.</t>
+          <t>SAU [DEV-207]: hồi quy đã sửa — `project.open` chạy XONG, trả `summary` 14 trường kèm `previous_session` và `tiep_tuc`. Nhưng `previous_session.summary` là `null`, nên nó KHÔNG thuật lại được quyết định nào đã chốt — đúng thứ đề bài hỏi.</t>
         </is>
       </c>
       <c r="K66" s="26" t="inlineStr">
@@ -6060,7 +6060,7 @@
       </c>
       <c r="M66" s="26" t="inlineStr">
         <is>
-          <t>Đây chính là điều anh báo trước đây: tác tử không biết việc đang dở là việc gì.</t>
+          <t>[DEV-203] cấp `project` = id làm `project.open` đi tìm `&lt;dự án&gt;/&lt;dự án&gt;` và hỏng E2000; [DEV-207] đổi sang đường dẫn tuyệt đối. Phần còn thiếu là NỘI DUNG khôi phục, không phải đường đi.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
[WI-TEST][DEV-213] Quyết định phạm vi: PCB và vai trò người dùng ngoài phạm vi v1.3
Chủ sản phẩm chốt 24/09/2026. Bộ 76 usecase đo một sản phẩm rộng hơn phạm vi
v1.3, nên vài ca hỏng vì CHƯA ĐỊNH LÀM, không vì LÀM SAI. Gọi một khoảng trống
phạm vi là lỗi thì bảng kết quả nói sai về sản phẩm: người đọc tưởng có thứ
hỏng cần sửa, trong khi thứ ấy chưa từng được hứa.

TC061 (hồ sơ sản xuất) và TC071 (vai trò người dùng) đổi sang nhãn 'Bỏ qua' —
nhãn mà chính sheet Huong dan dành cho trường hợp này — chứ không phải 'Bị
chặn' (môi trường kiểm thử thiếu) và cũng không phải 'Không đạt'.

Ranh giới vạch ở mức SƠ ĐỒ NGUYÊN LÝ: rà soát netlist/schematic và đối chiếu
BOM↔schematic vẫn trong phạm vi; chỉ phần mạch in đi ra.

Tìm kiếm: chốt SearXNG, tạm hoãn dựng. make searxng đã sẵn sàng; máy chủ công
cộng không dùng được (searx.be trả 200 với 0 kết quả, priv.au trả 429).

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Usecase_Test_Agent_Ky_Su_Nhung.xlsx
+++ b/docs/Usecase_Test_Agent_Ky_Su_Nhung.xlsx
@@ -5788,12 +5788,12 @@
       </c>
       <c r="I62" s="26" t="inlineStr">
         <is>
-          <t>Không đạt</t>
+          <t>Bỏ qua</t>
         </is>
       </c>
       <c r="J62" s="26" t="inlineStr">
         <is>
-          <t>Không xuất được hồ sơ sản xuất.</t>
+          <t>NGOÀI PHẠM VI v1.3 — chủ sản phẩm chốt 24/09/2026: phần PCB (bố trí mạch in, Gerber, drill, file gắp đặt, DRC) chưa làm trong sản phẩm này.</t>
         </is>
       </c>
       <c r="K62" s="26" t="inlineStr">
@@ -5808,7 +5808,7 @@
       </c>
       <c r="M62" s="26" t="inlineStr">
         <is>
-          <t>EIDE KHÔNG có năng lực layout PCB/Gerber/DRC nào trong 245 năng lực — đây là khoảng trống của sản phẩm, không phải lỗi lượt chạy.</t>
+          <t>Đổi nhãn từ “Không đạt” sang “Bỏ qua”: đây không phải lỗi, đây là thứ chưa định làm. Gọi một khoảng trống phạm vi là lỗi thì bảng kết quả nói sai về sản phẩm.</t>
         </is>
       </c>
     </row>
@@ -6430,12 +6430,12 @@
       </c>
       <c r="I72" s="26" t="inlineStr">
         <is>
-          <t>Bị chặn</t>
+          <t>Bỏ qua</t>
         </is>
       </c>
       <c r="J72" s="26" t="inlineStr">
         <is>
-          <t>Cần nhiều tài khoản người dùng có vai trò khác nhau.</t>
+          <t>NGOÀI PHẠM VI v1.3 — chủ sản phẩm chốt 24/09/2026: EIDE là ứng dụng một người trên máy cá nhân, không có khái niệm tài khoản hay vai trò.</t>
         </is>
       </c>
       <c r="K72" s="26" t="inlineStr">
@@ -6450,7 +6450,7 @@
       </c>
       <c r="M72" s="26" t="inlineStr">
         <is>
-          <t>EIDE không có khái niệm tài khoản hay vai trò — đây là KHOẢNG TRỐNG CỦA SẢN PHẨM, không phải thiếu sót của môi trường kiểm thử.</t>
+          <t>Trước đó ghi “Bị chặn (cần nhiều tài khoản)” — sai loại: không phải môi trường kiểm thử thiếu, mà là sản phẩm cố ý không có phần ấy.</t>
         </is>
       </c>
     </row>
@@ -6511,7 +6511,11 @@
           <t>23/09/2026</t>
         </is>
       </c>
-      <c r="M73" s="26" t="inlineStr"/>
+      <c r="M73" s="26" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> CHỜ CẤU HÌNH: `search.web` cần một máy chủ SearXNG; chủ sản phẩm chốt dùng SearXNG nhưng tạm hoãn dựng. `make searxng` đã sẵn sàng.</t>
+        </is>
+      </c>
     </row>
     <row r="74" ht="23.85" customHeight="1" s="16">
       <c r="A74" s="23" t="inlineStr">

</xml_diff>